<commit_message>
Add shortlist of 15 Austin real estate photography companies
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016XUjYcwbMrhJPcjoj1e8by
</commit_message>
<xml_diff>
--- a/austin-photographers/austin_photographers.xlsx
+++ b/austin-photographers/austin_photographers.xlsx
@@ -7,13 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="All" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Austin offices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RE shortlist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Austin offices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All'!$A$1:$P$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Austin offices'!$A$1:$P$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All'!$A$1:$P$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Austin offices'!$A$1:$P$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,6 +444,760 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Why picked</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Office status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Price hint</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>A Residential listings</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Boko Media</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Austin commercial office (Wild Basin Suite 250); since 2016; long hours (Mon-Sat); photo + drone + video + commercial</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>(512) 693-4021</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://bokomedia.com/</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>108 Wild Basin Rd S, Suite 250, Austin, TX 78746</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Commercial office/studio</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>https://bokomedia.com/contact/;https://www.bbb.org/us/tx/austin/profile/photographer/boko-media-real-estate-photography-video-0825-1000251207;https://www.yelp.com/biz/boko-media-austin</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>A Residential listings</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Come and Shoot It Photography</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cedar Park commercial office (Suite 501); since 2015; published pricing; the only one with a stated rating (5.0/29)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>(512) 400-4205</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.comeandshootitphotography.com/</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>1320 Arrow Point Dr, Ste 501, Cedar Park, TX 78613</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Commercial office/studio</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Pricing guide published on site</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.comeandshootitphotography.com/;https://www.comeandshootitphotography.com/real-estate-pricing-guide;https://www.yelp.com/biz/come-and-shoot-it-photography-cedar-park;https://local.yahoo.com/info-210266027-come-and-shoot-it-photography-cedar-park/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A Residential listings</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TK Images</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Since 2002 (oldest); Austin/Houston/San Antonio multi-city team; office hours M-F 9-5; published pricing</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>(512) 949-0988</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tkimages.com/locations/austin/</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>10301 Ranch to Market 2222 #712, Austin, TX 78730</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Address listed (type unclear)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Services &amp; Pricing page published</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tkimages.com/contact/;https://www.tkimages.com/locations/austin/;https://www.yelp.com/biz/tk-images-austin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>A Residential listings</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Austin 360 Photography</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Phone + email + pricing all published; full service line incl. commercial; named founder</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>(512) 686-4707</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>contact@austin360photography.com</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.austin360photography.com/</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Service-area only</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Pricing page published (austin360photography.com/pricing)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.austin360photography.com/contact/;https://www.austin360photography.com/pricing/;https://www.yelp.com/biz/austin-360-photography-austin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>A Residential listings</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Full Package Media</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Since 2017; claims tens of thousands of Austin homes shot; suited to high volume</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>(512) 910-8076</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://fullpackagemedia.com/locations/tx/austin-real-estate-photography/</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Service-area only</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Bundled pricing (details on site)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>https://fullpackagemedia.com/locations/tx/austin-real-estate-photography/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>A Residential listings</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Premier Property Productions</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Locally owned; fixed business hours; 512 local number</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>(512) 859-5200</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.premierpropertyproductions.com/</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Service-area only</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.premierpropertyproductions.com/;https://www.yelp.com/biz/premier-property-productions-austin</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>B Residential listings</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Real Image Pros</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Since 2015; covers both residential and architectural</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>(512) 474-7475</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.realimagepros.com/</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Service-area only</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.realimagepros.com/contact-3;https://www.thumbtack.com/tx/austin/real-estate-photographers/real-image-pros/service/361367751789133829</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>B Residential listings</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>ZABE Media</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Phone + email published; full service line (3D/floor plans/virtual staging)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>(512) 740-5445</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>contact@zabemedia.com</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://zabemedia.com/</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>3401 S Lamar Blvd, Austin, TX 78704</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Address listed (type unclear)</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://zabemedia.com/contact/;https://www.yellowpages.com/austin-tx/mip/zabe-media-579765910;https://www.yelp.com/biz/zabe-media-austin</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>B Residential listings</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Austin Real Estate Photography</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Clear pricing ($225 standard package) and turnaround (next day by 5pm); licensed and insured</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>(512) 914-8308</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://austinrealestatephotography.com/</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>5413 Link Ave, Austin, TX 78751</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Address listed (type unclear)</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>from $165 (STR) / $225 standard package</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://austinrealestatephotography.com/;https://www.yelp.com/biz/austin-real-estate-photography-austin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>B Residential listings</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Twist Tours</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Works with builders/architects; covers Austin + San Antonio; toll-free number + email</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>(866) 648-0022</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>info@twisttours.com</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.twisttours.com/</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>5102 Ridgemoor Dr, Austin, TX</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Address listed (type unclear)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.twisttours.com/contact-us/;https://www.yelp.com/biz/twist-tours-austin;https://www.twisttours.com/real-estate-photography/austin/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>B Residential listings</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Studio 12 Austin</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Since 2008; same-day delivery with no rush fee; online booking only (no phone found)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.studio12austin.com/</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Service-area only</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.studio12austin.com/;https://www.studio12austin.com/book-a-shoot.html;https://www.facebook.com/Studio12Austin/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>B Residential listings</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Virtuance</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>National standardized network, lowest price ($99/10 photos); good as a price benchmark or overflow capacity; weak local ties</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>(844) 443-7325</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.virtuance.com/austin-real-estate-photography/</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Service-area only</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>$99 / 10 photos; $149 / 25 photos</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.virtuance.com/austin-real-estate-photography/;https://www.virtuance.com/contact/;https://unifyrealestate.com/photography/virtuance/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>C Commercial/multifamily</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Justin Wallace Architecture Photography</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Austin commercial office; 15+ yrs; focuses on office/multifamily/commercial properties for brokers and property managers; 5.0 (15)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>(512) 814-8451</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>justin@justinwallacephotography.com</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.justinwallacephotography.com/</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>321 W Ben White Blvd, Ste 106A, Austin, TX 78704</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Commercial office/studio</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.justinwallacephotography.com/;https://www.yelp.com/biz/justin-wallace-austin;https://cars.superpages.com/austin-tx/bpp/justin-wallace-architecture-photography-538028493;https://reviews.birdeye.com/justin-wallace-photography-170416005248159</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>C Commercial/multifamily</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Images by Johnny Stevens</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Clients incl. American Campus Communities (student housing) and Michaels Org (multifamily); aerial; 5.0 (23)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>(512) 762-5621</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.johnnystevens.com/</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Austin, TX 78746 (Westlake)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Service-area only</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.johnnystevens.com/;https://www.johnnystevens.com/contact-johnny/;https://www.houzz.com/professionals/photographers/images-by-johnny-stevens-pfvwus-pf~1762556467;https://reviews.birdeye.com/images-by-johnny-stevens-166614963402006</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>C Commercial/multifamily</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Thomas McConnell Photography</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Clients incl. DPR Construction, Jacobs Engineering; high-end architecture/construction/healthcare projects; Tarrytown Center office</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>512-426-8368</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>tom@mcconnellphoto.net</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://mcconnellphoto.net/</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>2414 Exposition Blvd, Austin, TX 78703</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Commercial office/studio</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>https://mcconnellphoto.net/;https://www.yelp.com/biz/thomas-mcconnell-photography-austin;https://www.chamberofcommerce.com/business-directory/texas/austin/photographer/2028772842-thomas-mcconnell-photography;https://www.loopnet.com/Listing/2414-Exposition-Blvd-Austin-TX/14101395/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7444,7 +8199,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9135,7 +9890,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>